<commit_message>
bom and component sizing
</commit_message>
<xml_diff>
--- a/Manufacturing/ArduinoMegaEthernetBOM.xlsx
+++ b/Manufacturing/ArduinoMegaEthernetBOM.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="195">
   <si>
     <t>Arduino Mega with Ethernet</t>
   </si>
@@ -87,19 +87,19 @@
     <t>N/A</t>
   </si>
   <si>
-    <t>C44, C45</t>
+    <t>C1, C7-C9, C11, C12, C14-C19, C21, C22, C24-C27, C29, C32, C37, C40, C42, C47, C50</t>
   </si>
   <si>
-    <t>Murata Electronics</t>
+    <t>CCTC</t>
   </si>
   <si>
-    <t>GRM0335C1H120JA01D</t>
+    <t>TCC0603X7R104K250CT</t>
   </si>
   <si>
-    <t>CAP CER 12PF 50V C0G/NP0 0603</t>
+    <t>CAP CER 0.1UF 25V X7R 0603</t>
   </si>
   <si>
-    <t>0402 (1005 Metric)</t>
+    <t>C_0603_1608Metric</t>
   </si>
   <si>
     <t>SMD</t>
@@ -117,16 +117,13 @@
     <t>CAP CER 22PF 50V C0G/NP0 0603</t>
   </si>
   <si>
-    <t>C_0603_1608Metric</t>
-  </si>
-  <si>
     <t>C5, C13, C23, C35, C36, C38</t>
   </si>
   <si>
-    <t>GRM21BR61H106KE43L</t>
+    <t>TCC0805X5R106K500FT</t>
   </si>
   <si>
-    <t>CAP CER 10UF 50V X5R 0805</t>
+    <t>50V 10uF X5R ±10% 0805</t>
   </si>
   <si>
     <t>C_0805_2012Metric</t>
@@ -135,58 +132,22 @@
     <t>C6, C20, C34, C39, C41, C43, C46</t>
   </si>
   <si>
-    <t>Samsung Electro-Mechanics</t>
+    <t>TCC0603X7R105K160CT</t>
   </si>
   <si>
-    <t>CL10B105KP8NNNC</t>
-  </si>
-  <si>
-    <t>CAP CER 1UF 10V X7R 0603</t>
-  </si>
-  <si>
-    <t>C1, C7-C9, C11, C12, C14, C18, C24-C27, C29, C32, C37, C40, C42, C47</t>
-  </si>
-  <si>
-    <t>CL10B104KA8NNNC</t>
-  </si>
-  <si>
-    <t>CAP CER 0.1UF 25V X7R 0603</t>
+    <t>16V 1uF X7R ±10% 0603</t>
   </si>
   <si>
     <t>C10, C21</t>
+  </si>
+  <si>
+    <t>Murata Electronics</t>
   </si>
   <si>
     <t>GRM21BR71C475KE51K</t>
   </si>
   <si>
     <t>CAP CER 4.7UF 16V X7R 0805</t>
-  </si>
-  <si>
-    <t>C15, C16</t>
-  </si>
-  <si>
-    <t>CL10B682JB8NNNC</t>
-  </si>
-  <si>
-    <t>CAP CER 6800PF 50V X7R 0603</t>
-  </si>
-  <si>
-    <t>C17</t>
-  </si>
-  <si>
-    <t>CL10B223KB8WPNC</t>
-  </si>
-  <si>
-    <t>CAP CER 0.022UF 50V X7R 0603</t>
-  </si>
-  <si>
-    <t>C19, C22</t>
-  </si>
-  <si>
-    <t>CL10B103KB8NNNC</t>
-  </si>
-  <si>
-    <t>CAP CER 10000PF 50V X7R 0603</t>
   </si>
   <si>
     <t>C28, C30</t>
@@ -201,6 +162,9 @@
     <t>C31, C33, C48, C49</t>
   </si>
   <si>
+    <t>Samsung Electro-Mechanics</t>
+  </si>
+  <si>
     <t>CL31B226KPHNNNE</t>
   </si>
   <si>
@@ -210,34 +174,22 @@
     <t>C_0805_2012Metric_Pad1.18x1.45mm</t>
   </si>
   <si>
-    <t>D3</t>
+    <t>C44, C45</t>
   </si>
   <si>
-    <t>Lite-On Inc.</t>
+    <t>YAGEO</t>
   </si>
   <si>
-    <t>LTST-C190KFKT</t>
+    <t>CC0402JRNPO9BN120</t>
   </si>
   <si>
-    <t>LED ORANGE CLEAR CHIP SMD</t>
+    <t>CAP CER 12PF 50V C0G/NPO 0402</t>
   </si>
   <si>
-    <t>LED_0603_1608Metric</t>
-  </si>
-  <si>
-    <t>D5</t>
-  </si>
-  <si>
-    <t>LTST-C190GKT</t>
-  </si>
-  <si>
-    <t>LED GREEN CLEAR CHIP SMD</t>
+    <t>C_0402_1005Metric</t>
   </si>
   <si>
     <t>F1</t>
-  </si>
-  <si>
-    <t>YAGEO</t>
   </si>
   <si>
     <t>SMD1206B200TF</t>
@@ -249,7 +201,7 @@
     <t>Fuse_1206_3216Metric</t>
   </si>
   <si>
-    <t>FB1, FB2</t>
+    <t>FB1-FB4</t>
   </si>
   <si>
     <t>BLM18KG121TN1D</t>
@@ -264,10 +216,13 @@
     <t>J1</t>
   </si>
   <si>
-    <t>Amphenol ICC</t>
+    <t>WIZNET</t>
   </si>
   <si>
-    <t>RJMG1BD3B8K1ANR</t>
+    <t>RB1-125BAG1A</t>
+  </si>
+  <si>
+    <t>RJ45Receptacle 1 Shielded Right-Angle cat</t>
   </si>
   <si>
     <t>RJ45_Amphenol_RJMG1BD3B8K1ANR</t>
@@ -276,7 +231,10 @@
     <t>J2, J3, J4, J5, J6</t>
   </si>
   <si>
-    <t>Würth Elektronik</t>
+    <t>XFCN</t>
+  </si>
+  <si>
+    <t>PZ254V-11-03P</t>
   </si>
   <si>
     <t>CONN HEADER VERT 3POS 2.54MM</t>
@@ -286,6 +244,9 @@
   </si>
   <si>
     <t>J7</t>
+  </si>
+  <si>
+    <t>PZ254V-11-02P</t>
   </si>
   <si>
     <t>CONN HEADER VERT 2POS 2.54MM</t>
@@ -342,7 +303,10 @@
     <t>R1, R2, R6, R9, R10, R13</t>
   </si>
   <si>
-    <t>WR06X1002FTL</t>
+    <t>FOJAN</t>
+  </si>
+  <si>
+    <t>FRC0603F1002TS</t>
   </si>
   <si>
     <t>RES 10K OHM 1% 1/10W 0603</t>
@@ -399,61 +363,52 @@
     <t>R14-R16, R31, R32, R38-R40</t>
   </si>
   <si>
-    <t>RC0603FR-134K7L</t>
+    <t>FRC0603F4701TS</t>
   </si>
   <si>
     <t>RES 4.7K OHM 1% 1/10W 0603</t>
   </si>
   <si>
-    <t>R17-R20</t>
+    <t>R18, R20</t>
   </si>
   <si>
-    <t>RC0603FR-07330RL</t>
+    <t>RC0603FR-07470RL</t>
   </si>
   <si>
-    <t>RES 330 OHM 1% 1/10W 0603</t>
+    <t>RES 470 OHM 1% 1/10W 0603</t>
   </si>
   <si>
-    <t>R21</t>
-  </si>
-  <si>
-    <t>RC0603FR-0712K4L</t>
-  </si>
-  <si>
-    <t>RES 12.4K OHM 1% 1/10W 0603</t>
-  </si>
-  <si>
-    <t>R22</t>
-  </si>
-  <si>
-    <t>AC0603FR-0710RL</t>
-  </si>
-  <si>
-    <t>RES SMD 10 OHM 1% 1/10W 0603</t>
-  </si>
-  <si>
-    <t>R23, R25</t>
+    <t>R23, R25, R35, R36</t>
   </si>
   <si>
     <t>RC0603FR-0749R9L</t>
   </si>
   <si>
-    <t>R24, R26</t>
-  </si>
-  <si>
-    <t>RC0603FR-0782RL</t>
-  </si>
-  <si>
-    <t>RES 82 OHM 1% 1/10W 0603</t>
+    <t>RES 49.9R OHM 1% 1/10W 0603</t>
   </si>
   <si>
     <t>R27-R30</t>
   </si>
   <si>
-    <t>RT0603DRE0733RL</t>
+    <t>Vishay Intertech</t>
   </si>
   <si>
-    <t>RES SMD 33 OHM 0.5% 1/10W 0603</t>
+    <t>CRCW06033R30FKEAHP</t>
+  </si>
+  <si>
+    <t>±1% 3.3Ω 333mW 0603</t>
+  </si>
+  <si>
+    <t>R33</t>
+  </si>
+  <si>
+    <t>KOA Speer Electronics, Inc.</t>
+  </si>
+  <si>
+    <t>RN73R1JTTD1232F100</t>
+  </si>
+  <si>
+    <t>RES 12.3K OHM 1% 1/10W 0603</t>
   </si>
   <si>
     <t>SW1</t>
@@ -522,7 +477,7 @@
     <t>WIZnet</t>
   </si>
   <si>
-    <t>W5500</t>
+    <t>W6100-LQFP</t>
   </si>
   <si>
     <t>IC CTLR 3-1 ETH TCP/IP 48LQFP</t>
@@ -612,10 +567,10 @@
     <t>Y1</t>
   </si>
   <si>
-    <t>Jauch Quartz</t>
+    <t>YXC Crystal Oscillators</t>
   </si>
   <si>
-    <t>Q 16,0-JXS32-12-10/15-T1-WA-LF</t>
+    <t>X322516MOB4SI</t>
   </si>
   <si>
     <t>CRYSTAL 16.0000MHZ 12PF SMD</t>
@@ -653,13 +608,20 @@
   <si>
     <t>Total Cost Per Board:</t>
   </si>
+  <si>
+    <t>Manufacturing Cost:</t>
+  </si>
+  <si>
+    <t>Total:</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.000"/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -771,7 +733,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="30">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
@@ -838,11 +800,26 @@
     <xf borderId="1" fillId="4" fontId="5" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment vertical="bottom"/>
     </xf>
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" vertical="bottom"/>
+    </xf>
     <xf borderId="2" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="right" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="5" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="2" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="1" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="center"/>
@@ -1061,7 +1038,7 @@
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="9.0"/>
-    <col customWidth="1" min="2" max="2" width="71.43"/>
+    <col customWidth="1" min="2" max="2" width="86.0"/>
     <col customWidth="1" min="3" max="3" width="9.0"/>
     <col customWidth="1" min="4" max="4" width="27.86"/>
     <col customWidth="1" min="5" max="5" width="33.57"/>
@@ -1234,7 +1211,7 @@
         <v>0.12</v>
       </c>
       <c r="K5" s="14">
-        <f t="shared" ref="K5:K53" si="1">J5*C5</f>
+        <f t="shared" ref="K5:K46" si="1">J5*C5</f>
         <v>0.12</v>
       </c>
       <c r="L5" s="2"/>
@@ -1261,7 +1238,7 @@
         <v>19</v>
       </c>
       <c r="C6" s="11">
-        <v>2.0</v>
+        <v>25.0</v>
       </c>
       <c r="D6" s="12" t="s">
         <v>20</v>
@@ -1282,11 +1259,11 @@
         <v>18</v>
       </c>
       <c r="J6" s="15">
-        <v>0.1</v>
+        <v>0.0021</v>
       </c>
       <c r="K6" s="14">
         <f t="shared" si="1"/>
-        <v>0.2</v>
+        <v>0.0525</v>
       </c>
       <c r="L6" s="2"/>
       <c r="M6" s="2"/>
@@ -1312,7 +1289,7 @@
         <v>25</v>
       </c>
       <c r="C7" s="11">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="D7" s="12" t="s">
         <v>26</v>
@@ -1324,7 +1301,7 @@
         <v>28</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="H7" s="13" t="s">
         <v>24</v>
@@ -1337,7 +1314,7 @@
       </c>
       <c r="K7" s="14">
         <f t="shared" si="1"/>
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="L7" s="2"/>
       <c r="M7" s="2"/>
@@ -1360,7 +1337,7 @@
         <v>4.0</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C8" s="11">
         <v>6.0</v>
@@ -1369,13 +1346,13 @@
         <v>20</v>
       </c>
       <c r="E8" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="F8" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="F8" s="12" t="s">
+      <c r="G8" s="10" t="s">
         <v>32</v>
-      </c>
-      <c r="G8" s="10" t="s">
-        <v>33</v>
       </c>
       <c r="H8" s="13" t="s">
         <v>24</v>
@@ -1384,11 +1361,11 @@
         <v>18</v>
       </c>
       <c r="J8" s="15">
-        <v>0.165</v>
+        <v>0.0419</v>
       </c>
       <c r="K8" s="14">
         <f t="shared" si="1"/>
-        <v>0.99</v>
+        <v>0.2514</v>
       </c>
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>
@@ -1411,22 +1388,22 @@
         <v>5.0</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C9" s="11">
         <v>7.0</v>
       </c>
       <c r="D9" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="E9" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="F9" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="E9" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="F9" s="12" t="s">
-        <v>37</v>
-      </c>
       <c r="G9" s="10" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="H9" s="13" t="s">
         <v>24</v>
@@ -1435,11 +1412,11 @@
         <v>18</v>
       </c>
       <c r="J9" s="15">
-        <v>0.08</v>
+        <v>0.0039</v>
       </c>
       <c r="K9" s="14">
         <f t="shared" si="1"/>
-        <v>0.56</v>
+        <v>0.0273</v>
       </c>
       <c r="L9" s="2"/>
       <c r="M9" s="2"/>
@@ -1462,22 +1439,22 @@
         <v>6.0</v>
       </c>
       <c r="B10" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" s="11">
+        <v>2.0</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="E10" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="C10" s="11">
-        <v>18.0</v>
-      </c>
-      <c r="D10" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="E10" s="12" t="s">
+      <c r="F10" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="F10" s="12" t="s">
-        <v>40</v>
-      </c>
       <c r="G10" s="10" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="H10" s="13" t="s">
         <v>24</v>
@@ -1486,11 +1463,11 @@
         <v>18</v>
       </c>
       <c r="J10" s="15">
-        <v>0.08</v>
+        <v>0.12</v>
       </c>
       <c r="K10" s="14">
         <f t="shared" si="1"/>
-        <v>1.44</v>
+        <v>0.24</v>
       </c>
       <c r="L10" s="2"/>
       <c r="M10" s="2"/>
@@ -1513,22 +1490,22 @@
         <v>7.0</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C11" s="11">
         <v>2.0</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="E11" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="F11" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="F11" s="12" t="s">
-        <v>43</v>
-      </c>
       <c r="G11" s="10" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="H11" s="13" t="s">
         <v>24</v>
@@ -1537,11 +1514,11 @@
         <v>18</v>
       </c>
       <c r="J11" s="15">
-        <v>0.12</v>
+        <v>0.14</v>
       </c>
       <c r="K11" s="14">
         <f t="shared" si="1"/>
-        <v>0.24</v>
+        <v>0.28</v>
       </c>
       <c r="L11" s="2"/>
       <c r="M11" s="2"/>
@@ -1564,13 +1541,13 @@
         <v>8.0</v>
       </c>
       <c r="B12" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C12" s="11">
+        <v>4.0</v>
+      </c>
+      <c r="D12" s="12" t="s">
         <v>44</v>
-      </c>
-      <c r="C12" s="11">
-        <v>2.0</v>
-      </c>
-      <c r="D12" s="12" t="s">
-        <v>35</v>
       </c>
       <c r="E12" s="12" t="s">
         <v>45</v>
@@ -1579,7 +1556,7 @@
         <v>46</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>29</v>
+        <v>47</v>
       </c>
       <c r="H12" s="13" t="s">
         <v>24</v>
@@ -1588,11 +1565,11 @@
         <v>18</v>
       </c>
       <c r="J12" s="15">
-        <v>0.1</v>
+        <v>0.0655</v>
       </c>
       <c r="K12" s="14">
         <f t="shared" si="1"/>
-        <v>0.2</v>
+        <v>0.262</v>
       </c>
       <c r="L12" s="2"/>
       <c r="M12" s="2"/>
@@ -1615,22 +1592,22 @@
         <v>9.0</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C13" s="11">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F13" s="12" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>29</v>
+        <v>52</v>
       </c>
       <c r="H13" s="13" t="s">
         <v>24</v>
@@ -1639,11 +1616,11 @@
         <v>18</v>
       </c>
       <c r="J13" s="15">
-        <v>0.1</v>
+        <v>0.02</v>
       </c>
       <c r="K13" s="14">
         <f t="shared" si="1"/>
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="L13" s="2"/>
       <c r="M13" s="2"/>
@@ -1666,22 +1643,22 @@
         <v>10.0</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C14" s="11">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="F14" s="12" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>29</v>
+        <v>56</v>
       </c>
       <c r="H14" s="13" t="s">
         <v>24</v>
@@ -1690,11 +1667,11 @@
         <v>18</v>
       </c>
       <c r="J14" s="15">
-        <v>0.08</v>
+        <v>0.13</v>
       </c>
       <c r="K14" s="14">
         <f t="shared" si="1"/>
-        <v>0.16</v>
+        <v>0.13</v>
       </c>
       <c r="L14" s="2"/>
       <c r="M14" s="2"/>
@@ -1717,22 +1694,22 @@
         <v>11.0</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C15" s="11">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="F15" s="12" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>29</v>
+        <v>60</v>
       </c>
       <c r="H15" s="13" t="s">
         <v>24</v>
@@ -1741,11 +1718,11 @@
         <v>18</v>
       </c>
       <c r="J15" s="15">
-        <v>0.14</v>
+        <v>0.1</v>
       </c>
       <c r="K15" s="14">
         <f t="shared" si="1"/>
-        <v>0.28</v>
+        <v>0.4</v>
       </c>
       <c r="L15" s="2"/>
       <c r="M15" s="2"/>
@@ -1768,35 +1745,35 @@
         <v>12.0</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C16" s="11">
-        <v>4.0</v>
-      </c>
-      <c r="D16" s="12" t="s">
-        <v>35</v>
+        <v>1.0</v>
+      </c>
+      <c r="D16" s="10" t="s">
+        <v>62</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="F16" s="12" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="H16" s="13" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="I16" s="9" t="s">
         <v>18</v>
       </c>
       <c r="J16" s="15">
-        <v>0.39</v>
+        <v>3.4</v>
       </c>
       <c r="K16" s="14">
         <f t="shared" si="1"/>
-        <v>1.56</v>
+        <v>3.4</v>
       </c>
       <c r="L16" s="2"/>
       <c r="M16" s="2"/>
@@ -1819,22 +1796,22 @@
         <v>13.0</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="C17" s="11">
-        <v>1.0</v>
+        <v>5.0</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="F17" s="12" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="G17" s="10" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="H17" s="13" t="s">
         <v>24</v>
@@ -1843,11 +1820,11 @@
         <v>18</v>
       </c>
       <c r="J17" s="15">
-        <v>0.13</v>
+        <v>0.0149</v>
       </c>
       <c r="K17" s="14">
         <f t="shared" si="1"/>
-        <v>0.13</v>
+        <v>0.0745</v>
       </c>
       <c r="L17" s="2"/>
       <c r="M17" s="2"/>
@@ -1870,22 +1847,22 @@
         <v>14.0</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="C18" s="11">
         <v>1.0</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="H18" s="13" t="s">
         <v>24</v>
@@ -1894,11 +1871,11 @@
         <v>18</v>
       </c>
       <c r="J18" s="15">
-        <v>0.14</v>
+        <v>0.0131</v>
       </c>
       <c r="K18" s="14">
         <f t="shared" si="1"/>
-        <v>0.14</v>
+        <v>0.0131</v>
       </c>
       <c r="L18" s="2"/>
       <c r="M18" s="2"/>
@@ -1921,22 +1898,22 @@
         <v>15.0</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="C19" s="11">
         <v>1.0</v>
       </c>
-      <c r="D19" s="12" t="s">
-        <v>69</v>
+      <c r="D19" s="10" t="s">
+        <v>76</v>
       </c>
       <c r="E19" s="12" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="G19" s="10" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="H19" s="13" t="s">
         <v>24</v>
@@ -1945,11 +1922,11 @@
         <v>18</v>
       </c>
       <c r="J19" s="15">
-        <v>0.13</v>
+        <v>0.57</v>
       </c>
       <c r="K19" s="14">
         <f t="shared" si="1"/>
-        <v>0.13</v>
+        <v>0.57</v>
       </c>
       <c r="L19" s="2"/>
       <c r="M19" s="2"/>
@@ -1972,22 +1949,22 @@
         <v>16.0</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="C20" s="11">
-        <v>2.0</v>
-      </c>
-      <c r="D20" s="12" t="s">
-        <v>20</v>
+        <v>1.0</v>
+      </c>
+      <c r="D20" s="10" t="s">
+        <v>81</v>
       </c>
       <c r="E20" s="12" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="H20" s="13" t="s">
         <v>24</v>
@@ -1996,11 +1973,11 @@
         <v>18</v>
       </c>
       <c r="J20" s="15">
-        <v>0.1</v>
+        <v>2.66</v>
       </c>
       <c r="K20" s="14">
         <f t="shared" si="1"/>
-        <v>0.2</v>
+        <v>2.66</v>
       </c>
       <c r="L20" s="2"/>
       <c r="M20" s="2"/>
@@ -2023,35 +2000,35 @@
         <v>17.0</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="C21" s="11">
-        <v>1.0</v>
-      </c>
-      <c r="D21" s="10" t="s">
-        <v>78</v>
+        <v>2.0</v>
+      </c>
+      <c r="D21" s="16" t="s">
+        <v>86</v>
       </c>
       <c r="E21" s="12" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="F21" s="12" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="G21" s="10" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="H21" s="13" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="I21" s="9" t="s">
         <v>18</v>
       </c>
       <c r="J21" s="15">
-        <v>4.22</v>
+        <v>0.29</v>
       </c>
       <c r="K21" s="14">
         <f t="shared" si="1"/>
-        <v>4.22</v>
+        <v>0.58</v>
       </c>
       <c r="L21" s="2"/>
       <c r="M21" s="2"/>
@@ -2074,22 +2051,22 @@
         <v>18.0</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="C22" s="11">
-        <v>5.0</v>
+        <v>6.0</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="E22" s="12">
-        <v>6.1300311121E10</v>
+        <v>91</v>
+      </c>
+      <c r="E22" s="12" t="s">
+        <v>92</v>
       </c>
       <c r="F22" s="12" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="H22" s="13" t="s">
         <v>24</v>
@@ -2098,11 +2075,11 @@
         <v>18</v>
       </c>
       <c r="J22" s="15">
-        <v>0.12</v>
+        <v>9.0E-4</v>
       </c>
       <c r="K22" s="14">
         <f t="shared" si="1"/>
-        <v>0.6</v>
+        <v>0.0054</v>
       </c>
       <c r="L22" s="2"/>
       <c r="M22" s="2"/>
@@ -2125,22 +2102,22 @@
         <v>19.0</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="C23" s="11">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="D23" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="E23" s="12">
-        <v>6.1300211121E10</v>
+        <v>49</v>
+      </c>
+      <c r="E23" s="12" t="s">
+        <v>96</v>
       </c>
       <c r="F23" s="12" t="s">
-        <v>86</v>
+        <v>97</v>
       </c>
       <c r="G23" s="10" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="H23" s="13" t="s">
         <v>24</v>
@@ -2149,11 +2126,11 @@
         <v>18</v>
       </c>
       <c r="J23" s="15">
-        <v>0.12</v>
+        <v>0.1</v>
       </c>
       <c r="K23" s="14">
         <f t="shared" si="1"/>
-        <v>0.12</v>
+        <v>0.2</v>
       </c>
       <c r="L23" s="2"/>
       <c r="M23" s="2"/>
@@ -2176,22 +2153,22 @@
         <v>20.0</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="C24" s="11">
-        <v>1.0</v>
-      </c>
-      <c r="D24" s="10" t="s">
-        <v>89</v>
+        <v>3.0</v>
+      </c>
+      <c r="D24" s="12" t="s">
+        <v>49</v>
       </c>
       <c r="E24" s="12" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="F24" s="12" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="H24" s="13" t="s">
         <v>24</v>
@@ -2200,11 +2177,11 @@
         <v>18</v>
       </c>
       <c r="J24" s="15">
-        <v>0.57</v>
+        <v>0.009</v>
       </c>
       <c r="K24" s="14">
         <f t="shared" si="1"/>
-        <v>0.57</v>
+        <v>0.027</v>
       </c>
       <c r="L24" s="2"/>
       <c r="M24" s="2"/>
@@ -2227,35 +2204,29 @@
         <v>21.0</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="C25" s="11">
         <v>1.0</v>
       </c>
-      <c r="D25" s="10" t="s">
+      <c r="D25" s="17"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="G25" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="E25" s="12" t="s">
-        <v>95</v>
-      </c>
-      <c r="F25" s="12" t="s">
-        <v>96</v>
-      </c>
-      <c r="G25" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="H25" s="13" t="s">
+      <c r="H25" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="I25" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="J25" s="15">
-        <v>2.66</v>
-      </c>
+      <c r="I25" s="20" t="s">
+        <v>103</v>
+      </c>
+      <c r="J25" s="21"/>
       <c r="K25" s="14">
         <f t="shared" si="1"/>
-        <v>2.66</v>
+        <v>0</v>
       </c>
       <c r="L25" s="2"/>
       <c r="M25" s="2"/>
@@ -2278,22 +2249,22 @@
         <v>22.0</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="C26" s="11">
-        <v>2.0</v>
-      </c>
-      <c r="D26" s="16" t="s">
-        <v>99</v>
+        <v>1.0</v>
+      </c>
+      <c r="D26" s="12" t="s">
+        <v>49</v>
       </c>
       <c r="E26" s="12" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F26" s="12" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="H26" s="13" t="s">
         <v>24</v>
@@ -2302,11 +2273,11 @@
         <v>18</v>
       </c>
       <c r="J26" s="15">
-        <v>0.29</v>
+        <v>0.1</v>
       </c>
       <c r="K26" s="14">
         <f t="shared" si="1"/>
-        <v>0.58</v>
+        <v>0.1</v>
       </c>
       <c r="L26" s="2"/>
       <c r="M26" s="2"/>
@@ -2329,22 +2300,22 @@
         <v>23.0</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C27" s="11">
-        <v>6.0</v>
+        <v>1.0</v>
       </c>
       <c r="D27" s="12" t="s">
-        <v>69</v>
+        <v>49</v>
       </c>
       <c r="E27" s="12" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="F27" s="12" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="G27" s="10" t="s">
-        <v>106</v>
+        <v>94</v>
       </c>
       <c r="H27" s="13" t="s">
         <v>24</v>
@@ -2357,7 +2328,7 @@
       </c>
       <c r="K27" s="14">
         <f t="shared" si="1"/>
-        <v>0.6</v>
+        <v>0.1</v>
       </c>
       <c r="L27" s="2"/>
       <c r="M27" s="2"/>
@@ -2380,22 +2351,22 @@
         <v>24.0</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C28" s="11">
-        <v>2.0</v>
+        <v>8.0</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>69</v>
+        <v>91</v>
       </c>
       <c r="E28" s="12" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="F28" s="12" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>106</v>
+        <v>94</v>
       </c>
       <c r="H28" s="13" t="s">
         <v>24</v>
@@ -2404,11 +2375,11 @@
         <v>18</v>
       </c>
       <c r="J28" s="15">
-        <v>0.1</v>
+        <v>0.001</v>
       </c>
       <c r="K28" s="14">
         <f t="shared" si="1"/>
-        <v>0.2</v>
+        <v>0.008</v>
       </c>
       <c r="L28" s="2"/>
       <c r="M28" s="2"/>
@@ -2431,22 +2402,22 @@
         <v>25.0</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C29" s="11">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>69</v>
+        <v>49</v>
       </c>
       <c r="E29" s="12" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="F29" s="12" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="G29" s="10" t="s">
-        <v>106</v>
+        <v>94</v>
       </c>
       <c r="H29" s="13" t="s">
         <v>24</v>
@@ -2455,11 +2426,11 @@
         <v>18</v>
       </c>
       <c r="J29" s="15">
-        <v>0.1</v>
+        <v>0.0013</v>
       </c>
       <c r="K29" s="14">
         <f t="shared" si="1"/>
-        <v>0.3</v>
+        <v>0.0026</v>
       </c>
       <c r="L29" s="2"/>
       <c r="M29" s="2"/>
@@ -2482,29 +2453,35 @@
         <v>26.0</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="C30" s="11">
-        <v>1.0</v>
-      </c>
-      <c r="D30" s="17"/>
-      <c r="E30" s="17"/>
-      <c r="F30" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="G30" s="18" t="s">
-        <v>106</v>
-      </c>
-      <c r="H30" s="19" t="s">
+        <v>4.0</v>
+      </c>
+      <c r="D30" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="E30" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="F30" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="G30" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="H30" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="I30" s="20" t="s">
-        <v>115</v>
-      </c>
-      <c r="J30" s="21"/>
+      <c r="I30" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="J30" s="15">
+        <v>0.009</v>
+      </c>
       <c r="K30" s="14">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.036</v>
       </c>
       <c r="L30" s="2"/>
       <c r="M30" s="2"/>
@@ -2527,22 +2504,22 @@
         <v>27.0</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C31" s="11">
-        <v>1.0</v>
-      </c>
-      <c r="D31" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="E31" s="12" t="s">
-        <v>117</v>
-      </c>
-      <c r="F31" s="12" t="s">
-        <v>118</v>
+        <v>4.0</v>
+      </c>
+      <c r="D31" s="22" t="s">
+        <v>120</v>
+      </c>
+      <c r="E31" s="22" t="s">
+        <v>121</v>
+      </c>
+      <c r="F31" s="22" t="s">
+        <v>122</v>
       </c>
       <c r="G31" s="10" t="s">
-        <v>106</v>
+        <v>94</v>
       </c>
       <c r="H31" s="13" t="s">
         <v>24</v>
@@ -2551,11 +2528,11 @@
         <v>18</v>
       </c>
       <c r="J31" s="15">
-        <v>0.1</v>
+        <v>0.0911</v>
       </c>
       <c r="K31" s="14">
         <f t="shared" si="1"/>
-        <v>0.1</v>
+        <v>0.3644</v>
       </c>
       <c r="L31" s="2"/>
       <c r="M31" s="2"/>
@@ -2578,22 +2555,22 @@
         <v>28.0</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="C32" s="11">
         <v>1.0</v>
       </c>
-      <c r="D32" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="E32" s="12" t="s">
-        <v>120</v>
-      </c>
-      <c r="F32" s="12" t="s">
-        <v>121</v>
+      <c r="D32" s="23" t="s">
+        <v>124</v>
+      </c>
+      <c r="E32" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="F32" s="23" t="s">
+        <v>126</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>106</v>
+        <v>94</v>
       </c>
       <c r="H32" s="13" t="s">
         <v>24</v>
@@ -2629,22 +2606,22 @@
         <v>29.0</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="C33" s="11">
-        <v>8.0</v>
-      </c>
-      <c r="D33" s="12" t="s">
-        <v>69</v>
+        <v>1.0</v>
+      </c>
+      <c r="D33" s="16" t="s">
+        <v>128</v>
       </c>
       <c r="E33" s="12" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="F33" s="12" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="G33" s="10" t="s">
-        <v>106</v>
+        <v>131</v>
       </c>
       <c r="H33" s="13" t="s">
         <v>24</v>
@@ -2653,11 +2630,11 @@
         <v>18</v>
       </c>
       <c r="J33" s="15">
-        <v>0.1</v>
+        <v>0.1259</v>
       </c>
       <c r="K33" s="14">
         <f t="shared" si="1"/>
-        <v>0.8</v>
+        <v>0.1259</v>
       </c>
       <c r="L33" s="2"/>
       <c r="M33" s="2"/>
@@ -2680,22 +2657,22 @@
         <v>30.0</v>
       </c>
       <c r="B34" s="10" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="C34" s="11">
-        <v>4.0</v>
-      </c>
-      <c r="D34" s="12" t="s">
-        <v>69</v>
+        <v>1.0</v>
+      </c>
+      <c r="D34" s="16" t="s">
+        <v>133</v>
       </c>
       <c r="E34" s="12" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="F34" s="12" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="G34" s="10" t="s">
-        <v>106</v>
+        <v>136</v>
       </c>
       <c r="H34" s="13" t="s">
         <v>24</v>
@@ -2704,11 +2681,11 @@
         <v>18</v>
       </c>
       <c r="J34" s="15">
-        <v>0.1</v>
+        <v>12.71</v>
       </c>
       <c r="K34" s="14">
         <f t="shared" si="1"/>
-        <v>0.4</v>
+        <v>12.71</v>
       </c>
       <c r="L34" s="2"/>
       <c r="M34" s="2"/>
@@ -2731,22 +2708,22 @@
         <v>31.0</v>
       </c>
       <c r="B35" s="10" t="s">
-        <v>128</v>
+        <v>137</v>
       </c>
       <c r="C35" s="11">
         <v>1.0</v>
       </c>
-      <c r="D35" s="12" t="s">
-        <v>69</v>
+      <c r="D35" s="16" t="s">
+        <v>138</v>
       </c>
       <c r="E35" s="12" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="F35" s="12" t="s">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="G35" s="10" t="s">
-        <v>106</v>
+        <v>141</v>
       </c>
       <c r="H35" s="13" t="s">
         <v>24</v>
@@ -2755,11 +2732,11 @@
         <v>18</v>
       </c>
       <c r="J35" s="15">
-        <v>0.1</v>
+        <v>0.5242</v>
       </c>
       <c r="K35" s="14">
         <f t="shared" si="1"/>
-        <v>0.1</v>
+        <v>0.5242</v>
       </c>
       <c r="L35" s="2"/>
       <c r="M35" s="2"/>
@@ -2782,22 +2759,22 @@
         <v>32.0</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>131</v>
+        <v>142</v>
       </c>
       <c r="C36" s="11">
         <v>1.0</v>
       </c>
-      <c r="D36" s="12" t="s">
-        <v>69</v>
+      <c r="D36" s="16" t="s">
+        <v>143</v>
       </c>
       <c r="E36" s="12" t="s">
-        <v>132</v>
+        <v>144</v>
       </c>
       <c r="F36" s="12" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
       <c r="G36" s="10" t="s">
-        <v>106</v>
+        <v>146</v>
       </c>
       <c r="H36" s="13" t="s">
         <v>24</v>
@@ -2806,11 +2783,11 @@
         <v>18</v>
       </c>
       <c r="J36" s="15">
-        <v>0.1</v>
+        <v>6.564</v>
       </c>
       <c r="K36" s="14">
         <f t="shared" si="1"/>
-        <v>0.1</v>
+        <v>6.564</v>
       </c>
       <c r="L36" s="2"/>
       <c r="M36" s="2"/>
@@ -2833,22 +2810,22 @@
         <v>33.0</v>
       </c>
       <c r="B37" s="10" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
       <c r="C37" s="11">
-        <v>2.0</v>
-      </c>
-      <c r="D37" s="12" t="s">
-        <v>69</v>
+        <v>1.0</v>
+      </c>
+      <c r="D37" s="16" t="s">
+        <v>148</v>
       </c>
       <c r="E37" s="12" t="s">
-        <v>135</v>
+        <v>149</v>
       </c>
       <c r="F37" s="12" t="s">
-        <v>135</v>
+        <v>150</v>
       </c>
       <c r="G37" s="10" t="s">
-        <v>106</v>
+        <v>151</v>
       </c>
       <c r="H37" s="13" t="s">
         <v>24</v>
@@ -2857,11 +2834,11 @@
         <v>18</v>
       </c>
       <c r="J37" s="15">
-        <v>0.1</v>
+        <v>2.19</v>
       </c>
       <c r="K37" s="14">
         <f t="shared" si="1"/>
-        <v>0.2</v>
+        <v>2.19</v>
       </c>
       <c r="L37" s="2"/>
       <c r="M37" s="2"/>
@@ -2884,22 +2861,22 @@
         <v>34.0</v>
       </c>
       <c r="B38" s="10" t="s">
-        <v>136</v>
+        <v>152</v>
       </c>
       <c r="C38" s="11">
-        <v>2.0</v>
-      </c>
-      <c r="D38" s="12" t="s">
-        <v>69</v>
+        <v>1.0</v>
+      </c>
+      <c r="D38" s="16" t="s">
+        <v>153</v>
       </c>
       <c r="E38" s="12" t="s">
-        <v>137</v>
+        <v>154</v>
       </c>
       <c r="F38" s="12" t="s">
-        <v>138</v>
+        <v>155</v>
       </c>
       <c r="G38" s="10" t="s">
-        <v>106</v>
+        <v>156</v>
       </c>
       <c r="H38" s="13" t="s">
         <v>24</v>
@@ -2908,11 +2885,11 @@
         <v>18</v>
       </c>
       <c r="J38" s="15">
-        <v>0.1</v>
+        <v>0.96</v>
       </c>
       <c r="K38" s="14">
         <f t="shared" si="1"/>
-        <v>0.2</v>
+        <v>0.96</v>
       </c>
       <c r="L38" s="2"/>
       <c r="M38" s="2"/>
@@ -2935,22 +2912,22 @@
         <v>35.0</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>139</v>
+        <v>157</v>
       </c>
       <c r="C39" s="11">
-        <v>4.0</v>
-      </c>
-      <c r="D39" s="12" t="s">
-        <v>69</v>
+        <v>1.0</v>
+      </c>
+      <c r="D39" s="16" t="s">
+        <v>153</v>
       </c>
       <c r="E39" s="12" t="s">
-        <v>140</v>
+        <v>158</v>
       </c>
       <c r="F39" s="12" t="s">
-        <v>141</v>
+        <v>159</v>
       </c>
       <c r="G39" s="10" t="s">
-        <v>106</v>
+        <v>156</v>
       </c>
       <c r="H39" s="13" t="s">
         <v>24</v>
@@ -2959,11 +2936,11 @@
         <v>18</v>
       </c>
       <c r="J39" s="15">
-        <v>0.1</v>
+        <v>0.71</v>
       </c>
       <c r="K39" s="14">
         <f t="shared" si="1"/>
-        <v>0.4</v>
+        <v>0.71</v>
       </c>
       <c r="L39" s="2"/>
       <c r="M39" s="2"/>
@@ -2986,22 +2963,22 @@
         <v>36.0</v>
       </c>
       <c r="B40" s="10" t="s">
-        <v>142</v>
+        <v>160</v>
       </c>
       <c r="C40" s="11">
         <v>1.0</v>
       </c>
       <c r="D40" s="16" t="s">
-        <v>143</v>
+        <v>161</v>
       </c>
       <c r="E40" s="12" t="s">
-        <v>144</v>
+        <v>162</v>
       </c>
       <c r="F40" s="12" t="s">
-        <v>145</v>
+        <v>163</v>
       </c>
       <c r="G40" s="10" t="s">
-        <v>146</v>
+        <v>164</v>
       </c>
       <c r="H40" s="13" t="s">
         <v>24</v>
@@ -3010,11 +2987,11 @@
         <v>18</v>
       </c>
       <c r="J40" s="15">
-        <v>0.41</v>
+        <v>5.19</v>
       </c>
       <c r="K40" s="14">
         <f t="shared" si="1"/>
-        <v>0.41</v>
+        <v>5.19</v>
       </c>
       <c r="L40" s="2"/>
       <c r="M40" s="2"/>
@@ -3037,22 +3014,22 @@
         <v>37.0</v>
       </c>
       <c r="B41" s="10" t="s">
-        <v>147</v>
+        <v>165</v>
       </c>
       <c r="C41" s="11">
         <v>1.0</v>
       </c>
       <c r="D41" s="16" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="E41" s="12" t="s">
-        <v>149</v>
+        <v>166</v>
       </c>
       <c r="F41" s="12" t="s">
-        <v>150</v>
+        <v>167</v>
       </c>
       <c r="G41" s="10" t="s">
-        <v>151</v>
+        <v>168</v>
       </c>
       <c r="H41" s="13" t="s">
         <v>24</v>
@@ -3061,11 +3038,11 @@
         <v>18</v>
       </c>
       <c r="J41" s="15">
-        <v>17.3</v>
+        <v>0.35</v>
       </c>
       <c r="K41" s="14">
         <f t="shared" si="1"/>
-        <v>17.3</v>
+        <v>0.35</v>
       </c>
       <c r="L41" s="2"/>
       <c r="M41" s="2"/>
@@ -3088,22 +3065,22 @@
         <v>38.0</v>
       </c>
       <c r="B42" s="10" t="s">
-        <v>152</v>
+        <v>169</v>
       </c>
       <c r="C42" s="11">
         <v>1.0</v>
       </c>
       <c r="D42" s="16" t="s">
-        <v>153</v>
+        <v>133</v>
       </c>
       <c r="E42" s="12" t="s">
-        <v>154</v>
+        <v>170</v>
       </c>
       <c r="F42" s="12" t="s">
-        <v>155</v>
+        <v>171</v>
       </c>
       <c r="G42" s="10" t="s">
-        <v>156</v>
+        <v>172</v>
       </c>
       <c r="H42" s="13" t="s">
         <v>24</v>
@@ -3112,11 +3089,11 @@
         <v>18</v>
       </c>
       <c r="J42" s="15">
-        <v>0.5242</v>
+        <v>0.97</v>
       </c>
       <c r="K42" s="14">
         <f t="shared" si="1"/>
-        <v>0.5242</v>
+        <v>0.97</v>
       </c>
       <c r="L42" s="2"/>
       <c r="M42" s="2"/>
@@ -3139,22 +3116,22 @@
         <v>39.0</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>157</v>
+        <v>173</v>
       </c>
       <c r="C43" s="11">
         <v>1.0</v>
       </c>
       <c r="D43" s="16" t="s">
-        <v>158</v>
+        <v>174</v>
       </c>
       <c r="E43" s="12" t="s">
-        <v>159</v>
+        <v>175</v>
       </c>
       <c r="F43" s="12" t="s">
-        <v>160</v>
+        <v>176</v>
       </c>
       <c r="G43" s="10" t="s">
-        <v>161</v>
+        <v>177</v>
       </c>
       <c r="H43" s="13" t="s">
         <v>24</v>
@@ -3163,11 +3140,11 @@
         <v>18</v>
       </c>
       <c r="J43" s="15">
-        <v>6.564</v>
+        <v>0.2234</v>
       </c>
       <c r="K43" s="14">
         <f t="shared" si="1"/>
-        <v>6.564</v>
+        <v>0.2234</v>
       </c>
       <c r="L43" s="2"/>
       <c r="M43" s="2"/>
@@ -3190,22 +3167,22 @@
         <v>40.0</v>
       </c>
       <c r="B44" s="10" t="s">
-        <v>162</v>
+        <v>178</v>
       </c>
       <c r="C44" s="11">
         <v>1.0</v>
       </c>
       <c r="D44" s="16" t="s">
-        <v>163</v>
+        <v>179</v>
       </c>
       <c r="E44" s="12" t="s">
-        <v>164</v>
+        <v>180</v>
       </c>
       <c r="F44" s="12" t="s">
-        <v>165</v>
+        <v>181</v>
       </c>
       <c r="G44" s="10" t="s">
-        <v>166</v>
+        <v>182</v>
       </c>
       <c r="H44" s="13" t="s">
         <v>24</v>
@@ -3214,11 +3191,11 @@
         <v>18</v>
       </c>
       <c r="J44" s="15">
-        <v>3.6</v>
+        <v>0.0609</v>
       </c>
       <c r="K44" s="14">
         <f t="shared" si="1"/>
-        <v>3.6</v>
+        <v>0.0609</v>
       </c>
       <c r="L44" s="2"/>
       <c r="M44" s="2"/>
@@ -3241,22 +3218,22 @@
         <v>41.0</v>
       </c>
       <c r="B45" s="10" t="s">
-        <v>167</v>
+        <v>183</v>
       </c>
       <c r="C45" s="11">
         <v>1.0</v>
       </c>
       <c r="D45" s="16" t="s">
-        <v>168</v>
+        <v>184</v>
       </c>
       <c r="E45" s="12" t="s">
-        <v>169</v>
+        <v>185</v>
       </c>
       <c r="F45" s="12" t="s">
-        <v>170</v>
+        <v>186</v>
       </c>
       <c r="G45" s="10" t="s">
-        <v>171</v>
+        <v>182</v>
       </c>
       <c r="H45" s="13" t="s">
         <v>24</v>
@@ -3265,11 +3242,11 @@
         <v>18</v>
       </c>
       <c r="J45" s="15">
-        <v>0.96</v>
+        <v>0.23</v>
       </c>
       <c r="K45" s="14">
         <f t="shared" si="1"/>
-        <v>0.96</v>
+        <v>0.23</v>
       </c>
       <c r="L45" s="2"/>
       <c r="M45" s="2"/>
@@ -3292,22 +3269,22 @@
         <v>42.0</v>
       </c>
       <c r="B46" s="10" t="s">
-        <v>172</v>
+        <v>187</v>
       </c>
       <c r="C46" s="11">
         <v>1.0</v>
       </c>
       <c r="D46" s="16" t="s">
-        <v>168</v>
+        <v>188</v>
       </c>
       <c r="E46" s="12" t="s">
-        <v>173</v>
+        <v>189</v>
       </c>
       <c r="F46" s="12" t="s">
-        <v>174</v>
+        <v>190</v>
       </c>
       <c r="G46" s="10" t="s">
-        <v>171</v>
+        <v>191</v>
       </c>
       <c r="H46" s="13" t="s">
         <v>24</v>
@@ -3316,11 +3293,11 @@
         <v>18</v>
       </c>
       <c r="J46" s="15">
-        <v>0.71</v>
+        <v>0.28</v>
       </c>
       <c r="K46" s="14">
         <f t="shared" si="1"/>
-        <v>0.71</v>
+        <v>0.28</v>
       </c>
       <c r="L46" s="2"/>
       <c r="M46" s="2"/>
@@ -3339,40 +3316,12 @@
       <c r="Z46" s="2"/>
     </row>
     <row r="47" ht="14.25" customHeight="1">
-      <c r="A47" s="9">
-        <v>43.0</v>
-      </c>
-      <c r="B47" s="10" t="s">
-        <v>175</v>
-      </c>
-      <c r="C47" s="11">
-        <v>1.0</v>
-      </c>
-      <c r="D47" s="16" t="s">
-        <v>176</v>
-      </c>
-      <c r="E47" s="12" t="s">
-        <v>177</v>
-      </c>
-      <c r="F47" s="12" t="s">
-        <v>178</v>
-      </c>
-      <c r="G47" s="10" t="s">
-        <v>179</v>
-      </c>
-      <c r="H47" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="I47" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="J47" s="15">
-        <v>5.19</v>
-      </c>
-      <c r="K47" s="14">
-        <f t="shared" si="1"/>
-        <v>5.19</v>
-      </c>
+      <c r="F47" s="2"/>
+      <c r="G47" s="2"/>
+      <c r="H47" s="2"/>
+      <c r="I47" s="2"/>
+      <c r="J47" s="2"/>
+      <c r="K47" s="2"/>
       <c r="L47" s="2"/>
       <c r="M47" s="2"/>
       <c r="N47" s="2"/>
@@ -3390,39 +3339,16 @@
       <c r="Z47" s="2"/>
     </row>
     <row r="48" ht="14.25" customHeight="1">
-      <c r="A48" s="9">
-        <v>44.0</v>
-      </c>
-      <c r="B48" s="10" t="s">
-        <v>180</v>
-      </c>
-      <c r="C48" s="11">
-        <v>1.0</v>
-      </c>
-      <c r="D48" s="16" t="s">
-        <v>168</v>
-      </c>
-      <c r="E48" s="12" t="s">
-        <v>181</v>
-      </c>
-      <c r="F48" s="12" t="s">
-        <v>182</v>
-      </c>
-      <c r="G48" s="10" t="s">
-        <v>183</v>
-      </c>
-      <c r="H48" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="I48" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="J48" s="15">
-        <v>0.35</v>
-      </c>
-      <c r="K48" s="14">
-        <f t="shared" si="1"/>
-        <v>0.35</v>
+      <c r="F48" s="2"/>
+      <c r="G48" s="2"/>
+      <c r="H48" s="2"/>
+      <c r="I48" s="24" t="s">
+        <v>192</v>
+      </c>
+      <c r="J48" s="25"/>
+      <c r="K48" s="26">
+        <f>SUM(K2:K46)</f>
+        <v>41.4326</v>
       </c>
       <c r="L48" s="2"/>
       <c r="M48" s="2"/>
@@ -3441,39 +3367,15 @@
       <c r="Z48" s="2"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
-      <c r="A49" s="9">
-        <v>45.0</v>
-      </c>
-      <c r="B49" s="10" t="s">
-        <v>184</v>
-      </c>
-      <c r="C49" s="11">
+      <c r="F49" s="2"/>
+      <c r="G49" s="2"/>
+      <c r="H49" s="2"/>
+      <c r="I49" s="27" t="s">
+        <v>193</v>
+      </c>
+      <c r="J49" s="25"/>
+      <c r="K49" s="26">
         <v>1.0</v>
-      </c>
-      <c r="D49" s="16" t="s">
-        <v>148</v>
-      </c>
-      <c r="E49" s="12" t="s">
-        <v>185</v>
-      </c>
-      <c r="F49" s="12" t="s">
-        <v>186</v>
-      </c>
-      <c r="G49" s="10" t="s">
-        <v>187</v>
-      </c>
-      <c r="H49" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="I49" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="J49" s="15">
-        <v>0.97</v>
-      </c>
-      <c r="K49" s="14">
-        <f t="shared" si="1"/>
-        <v>0.97</v>
       </c>
       <c r="L49" s="2"/>
       <c r="M49" s="2"/>
@@ -3492,39 +3394,16 @@
       <c r="Z49" s="2"/>
     </row>
     <row r="50" ht="14.25" customHeight="1">
-      <c r="A50" s="9">
-        <v>46.0</v>
-      </c>
-      <c r="B50" s="10" t="s">
-        <v>188</v>
-      </c>
-      <c r="C50" s="11">
-        <v>1.0</v>
-      </c>
-      <c r="D50" s="16" t="s">
-        <v>189</v>
-      </c>
-      <c r="E50" s="12" t="s">
-        <v>190</v>
-      </c>
-      <c r="F50" s="12" t="s">
-        <v>191</v>
-      </c>
-      <c r="G50" s="10" t="s">
-        <v>192</v>
-      </c>
-      <c r="H50" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="I50" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="J50" s="15">
-        <v>1.25</v>
-      </c>
-      <c r="K50" s="14">
-        <f t="shared" si="1"/>
-        <v>1.25</v>
+      <c r="F50" s="2"/>
+      <c r="G50" s="2"/>
+      <c r="H50" s="2"/>
+      <c r="I50" s="2"/>
+      <c r="J50" s="28" t="s">
+        <v>194</v>
+      </c>
+      <c r="K50" s="26">
+        <f>K48+K49</f>
+        <v>42.4326</v>
       </c>
       <c r="L50" s="2"/>
       <c r="M50" s="2"/>
@@ -3543,40 +3422,12 @@
       <c r="Z50" s="2"/>
     </row>
     <row r="51" ht="14.25" customHeight="1">
-      <c r="A51" s="9">
-        <v>47.0</v>
-      </c>
-      <c r="B51" s="10" t="s">
-        <v>193</v>
-      </c>
-      <c r="C51" s="11">
-        <v>1.0</v>
-      </c>
-      <c r="D51" s="16" t="s">
-        <v>194</v>
-      </c>
-      <c r="E51" s="12" t="s">
-        <v>195</v>
-      </c>
-      <c r="F51" s="12" t="s">
-        <v>196</v>
-      </c>
-      <c r="G51" s="10" t="s">
-        <v>197</v>
-      </c>
-      <c r="H51" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="I51" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="J51" s="15">
-        <v>0.64</v>
-      </c>
-      <c r="K51" s="14">
-        <f t="shared" si="1"/>
-        <v>0.64</v>
-      </c>
+      <c r="F51" s="2"/>
+      <c r="G51" s="2"/>
+      <c r="H51" s="2"/>
+      <c r="I51" s="2"/>
+      <c r="J51" s="2"/>
+      <c r="K51" s="2"/>
       <c r="L51" s="2"/>
       <c r="M51" s="2"/>
       <c r="N51" s="2"/>
@@ -3594,40 +3445,12 @@
       <c r="Z51" s="2"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
-      <c r="A52" s="9">
-        <v>48.0</v>
-      </c>
-      <c r="B52" s="10" t="s">
-        <v>198</v>
-      </c>
-      <c r="C52" s="11">
-        <v>1.0</v>
-      </c>
-      <c r="D52" s="16" t="s">
-        <v>199</v>
-      </c>
-      <c r="E52" s="12" t="s">
-        <v>200</v>
-      </c>
-      <c r="F52" s="12" t="s">
-        <v>201</v>
-      </c>
-      <c r="G52" s="10" t="s">
-        <v>197</v>
-      </c>
-      <c r="H52" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="I52" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="J52" s="15">
-        <v>0.23</v>
-      </c>
-      <c r="K52" s="14">
-        <f t="shared" si="1"/>
-        <v>0.23</v>
-      </c>
+      <c r="F52" s="2"/>
+      <c r="G52" s="2"/>
+      <c r="H52" s="2"/>
+      <c r="I52" s="2"/>
+      <c r="J52" s="2"/>
+      <c r="K52" s="2"/>
       <c r="L52" s="2"/>
       <c r="M52" s="2"/>
       <c r="N52" s="2"/>
@@ -3645,40 +3468,12 @@
       <c r="Z52" s="2"/>
     </row>
     <row r="53" ht="14.25" customHeight="1">
-      <c r="A53" s="9">
-        <v>49.0</v>
-      </c>
-      <c r="B53" s="10" t="s">
-        <v>202</v>
-      </c>
-      <c r="C53" s="11">
-        <v>1.0</v>
-      </c>
-      <c r="D53" s="16" t="s">
-        <v>203</v>
-      </c>
-      <c r="E53" s="12" t="s">
-        <v>204</v>
-      </c>
-      <c r="F53" s="12" t="s">
-        <v>205</v>
-      </c>
-      <c r="G53" s="10" t="s">
-        <v>206</v>
-      </c>
-      <c r="H53" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="I53" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="J53" s="15">
-        <v>0.28</v>
-      </c>
-      <c r="K53" s="14">
-        <f t="shared" si="1"/>
-        <v>0.28</v>
-      </c>
+      <c r="F53" s="2"/>
+      <c r="G53" s="2"/>
+      <c r="H53" s="2"/>
+      <c r="I53" s="2"/>
+      <c r="J53" s="2"/>
+      <c r="K53" s="2"/>
       <c r="L53" s="2"/>
       <c r="M53" s="2"/>
       <c r="N53" s="2"/>
@@ -3722,14 +3517,9 @@
       <c r="F55" s="2"/>
       <c r="G55" s="2"/>
       <c r="H55" s="2"/>
-      <c r="I55" s="22" t="s">
-        <v>207</v>
-      </c>
-      <c r="J55" s="23"/>
-      <c r="K55" s="14">
-        <f>SUM(K2:K53)</f>
-        <v>57.8782</v>
-      </c>
+      <c r="I55" s="2"/>
+      <c r="J55" s="2"/>
+      <c r="K55" s="2"/>
       <c r="L55" s="2"/>
       <c r="M55" s="2"/>
       <c r="N55" s="2"/>
@@ -3816,6 +3606,11 @@
       <c r="Z58" s="2"/>
     </row>
     <row r="59" ht="14.25" customHeight="1">
+      <c r="A59" s="2"/>
+      <c r="B59" s="2"/>
+      <c r="C59" s="2"/>
+      <c r="D59" s="2"/>
+      <c r="E59" s="2"/>
       <c r="F59" s="2"/>
       <c r="G59" s="2"/>
       <c r="H59" s="2"/>
@@ -3839,6 +3634,11 @@
       <c r="Z59" s="2"/>
     </row>
     <row r="60" ht="14.25" customHeight="1">
+      <c r="A60" s="2"/>
+      <c r="B60" s="2"/>
+      <c r="C60" s="2"/>
+      <c r="D60" s="2"/>
+      <c r="E60" s="2"/>
       <c r="F60" s="2"/>
       <c r="G60" s="2"/>
       <c r="H60" s="2"/>
@@ -3862,6 +3662,11 @@
       <c r="Z60" s="2"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
+      <c r="A61" s="2"/>
+      <c r="B61" s="2"/>
+      <c r="C61" s="2"/>
+      <c r="D61" s="2"/>
+      <c r="E61" s="2"/>
       <c r="F61" s="2"/>
       <c r="G61" s="2"/>
       <c r="H61" s="2"/>
@@ -3885,6 +3690,11 @@
       <c r="Z61" s="2"/>
     </row>
     <row r="62" ht="14.25" customHeight="1">
+      <c r="A62" s="2"/>
+      <c r="B62" s="2"/>
+      <c r="C62" s="2"/>
+      <c r="D62" s="2"/>
+      <c r="E62" s="2"/>
       <c r="F62" s="2"/>
       <c r="G62" s="2"/>
       <c r="H62" s="2"/>
@@ -3908,6 +3718,11 @@
       <c r="Z62" s="2"/>
     </row>
     <row r="63" ht="14.25" customHeight="1">
+      <c r="A63" s="2"/>
+      <c r="B63" s="2"/>
+      <c r="C63" s="2"/>
+      <c r="D63" s="2"/>
+      <c r="E63" s="2"/>
       <c r="F63" s="2"/>
       <c r="G63" s="2"/>
       <c r="H63" s="2"/>
@@ -3931,6 +3746,11 @@
       <c r="Z63" s="2"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
+      <c r="A64" s="2"/>
+      <c r="B64" s="2"/>
+      <c r="C64" s="2"/>
+      <c r="D64" s="2"/>
+      <c r="E64" s="2"/>
       <c r="F64" s="2"/>
       <c r="G64" s="2"/>
       <c r="H64" s="2"/>
@@ -3954,6 +3774,11 @@
       <c r="Z64" s="2"/>
     </row>
     <row r="65" ht="14.25" customHeight="1">
+      <c r="A65" s="2"/>
+      <c r="B65" s="2"/>
+      <c r="C65" s="2"/>
+      <c r="D65" s="2"/>
+      <c r="E65" s="2"/>
       <c r="F65" s="2"/>
       <c r="G65" s="2"/>
       <c r="H65" s="2"/>
@@ -4313,11 +4138,11 @@
       <c r="Z77" s="2"/>
     </row>
     <row r="78" ht="14.25" customHeight="1">
-      <c r="A78" s="2"/>
-      <c r="B78" s="2"/>
-      <c r="C78" s="2"/>
-      <c r="D78" s="2"/>
-      <c r="E78" s="2"/>
+      <c r="A78" s="29"/>
+      <c r="B78" s="29"/>
+      <c r="C78" s="29"/>
+      <c r="D78" s="29"/>
+      <c r="E78" s="29"/>
       <c r="F78" s="2"/>
       <c r="G78" s="2"/>
       <c r="H78" s="2"/>
@@ -4341,11 +4166,11 @@
       <c r="Z78" s="2"/>
     </row>
     <row r="79" ht="14.25" customHeight="1">
-      <c r="A79" s="2"/>
-      <c r="B79" s="2"/>
-      <c r="C79" s="2"/>
-      <c r="D79" s="2"/>
-      <c r="E79" s="2"/>
+      <c r="A79" s="29"/>
+      <c r="B79" s="29"/>
+      <c r="C79" s="29"/>
+      <c r="D79" s="29"/>
+      <c r="E79" s="29"/>
       <c r="F79" s="2"/>
       <c r="G79" s="2"/>
       <c r="H79" s="2"/>
@@ -4369,11 +4194,11 @@
       <c r="Z79" s="2"/>
     </row>
     <row r="80" ht="14.25" customHeight="1">
-      <c r="A80" s="2"/>
-      <c r="B80" s="2"/>
-      <c r="C80" s="2"/>
-      <c r="D80" s="2"/>
-      <c r="E80" s="2"/>
+      <c r="A80" s="29"/>
+      <c r="B80" s="29"/>
+      <c r="C80" s="29"/>
+      <c r="D80" s="29"/>
+      <c r="E80" s="29"/>
       <c r="F80" s="2"/>
       <c r="G80" s="2"/>
       <c r="H80" s="2"/>
@@ -4397,11 +4222,11 @@
       <c r="Z80" s="2"/>
     </row>
     <row r="81" ht="14.25" customHeight="1">
-      <c r="A81" s="2"/>
-      <c r="B81" s="2"/>
-      <c r="C81" s="2"/>
-      <c r="D81" s="2"/>
-      <c r="E81" s="2"/>
+      <c r="A81" s="29"/>
+      <c r="B81" s="29"/>
+      <c r="C81" s="29"/>
+      <c r="D81" s="29"/>
+      <c r="E81" s="29"/>
       <c r="F81" s="2"/>
       <c r="G81" s="2"/>
       <c r="H81" s="2"/>
@@ -4425,11 +4250,11 @@
       <c r="Z81" s="2"/>
     </row>
     <row r="82" ht="14.25" customHeight="1">
-      <c r="A82" s="2"/>
-      <c r="B82" s="2"/>
-      <c r="C82" s="2"/>
-      <c r="D82" s="2"/>
-      <c r="E82" s="2"/>
+      <c r="A82" s="29"/>
+      <c r="B82" s="29"/>
+      <c r="C82" s="29"/>
+      <c r="D82" s="29"/>
+      <c r="E82" s="29"/>
       <c r="F82" s="2"/>
       <c r="G82" s="2"/>
       <c r="H82" s="2"/>
@@ -4453,11 +4278,11 @@
       <c r="Z82" s="2"/>
     </row>
     <row r="83" ht="14.25" customHeight="1">
-      <c r="A83" s="2"/>
-      <c r="B83" s="2"/>
-      <c r="C83" s="2"/>
-      <c r="D83" s="2"/>
-      <c r="E83" s="2"/>
+      <c r="A83" s="29"/>
+      <c r="B83" s="29"/>
+      <c r="C83" s="29"/>
+      <c r="D83" s="29"/>
+      <c r="E83" s="29"/>
       <c r="F83" s="2"/>
       <c r="G83" s="2"/>
       <c r="H83" s="2"/>
@@ -4481,11 +4306,11 @@
       <c r="Z83" s="2"/>
     </row>
     <row r="84" ht="14.25" customHeight="1">
-      <c r="A84" s="2"/>
-      <c r="B84" s="2"/>
-      <c r="C84" s="2"/>
-      <c r="D84" s="2"/>
-      <c r="E84" s="2"/>
+      <c r="A84" s="29"/>
+      <c r="B84" s="29"/>
+      <c r="C84" s="29"/>
+      <c r="D84" s="29"/>
+      <c r="E84" s="29"/>
       <c r="F84" s="2"/>
       <c r="G84" s="2"/>
       <c r="H84" s="2"/>
@@ -4509,11 +4334,11 @@
       <c r="Z84" s="2"/>
     </row>
     <row r="85" ht="14.25" customHeight="1">
-      <c r="A85" s="24"/>
-      <c r="B85" s="24"/>
-      <c r="C85" s="24"/>
-      <c r="D85" s="24"/>
-      <c r="E85" s="24"/>
+      <c r="A85" s="29"/>
+      <c r="B85" s="29"/>
+      <c r="C85" s="29"/>
+      <c r="D85" s="29"/>
+      <c r="E85" s="29"/>
       <c r="F85" s="2"/>
       <c r="G85" s="2"/>
       <c r="H85" s="2"/>
@@ -4537,11 +4362,11 @@
       <c r="Z85" s="2"/>
     </row>
     <row r="86" ht="14.25" customHeight="1">
-      <c r="A86" s="24"/>
-      <c r="B86" s="24"/>
-      <c r="C86" s="24"/>
-      <c r="D86" s="24"/>
-      <c r="E86" s="24"/>
+      <c r="A86" s="29"/>
+      <c r="B86" s="29"/>
+      <c r="C86" s="29"/>
+      <c r="D86" s="29"/>
+      <c r="E86" s="29"/>
       <c r="F86" s="2"/>
       <c r="G86" s="2"/>
       <c r="H86" s="2"/>
@@ -4565,11 +4390,11 @@
       <c r="Z86" s="2"/>
     </row>
     <row r="87" ht="14.25" customHeight="1">
-      <c r="A87" s="24"/>
-      <c r="B87" s="24"/>
-      <c r="C87" s="24"/>
-      <c r="D87" s="24"/>
-      <c r="E87" s="24"/>
+      <c r="A87" s="29"/>
+      <c r="B87" s="29"/>
+      <c r="C87" s="29"/>
+      <c r="D87" s="29"/>
+      <c r="E87" s="29"/>
       <c r="F87" s="2"/>
       <c r="G87" s="2"/>
       <c r="H87" s="2"/>
@@ -4593,11 +4418,11 @@
       <c r="Z87" s="2"/>
     </row>
     <row r="88" ht="14.25" customHeight="1">
-      <c r="A88" s="24"/>
-      <c r="B88" s="24"/>
-      <c r="C88" s="24"/>
-      <c r="D88" s="24"/>
-      <c r="E88" s="24"/>
+      <c r="A88" s="29"/>
+      <c r="B88" s="29"/>
+      <c r="C88" s="29"/>
+      <c r="D88" s="29"/>
+      <c r="E88" s="29"/>
       <c r="F88" s="2"/>
       <c r="G88" s="2"/>
       <c r="H88" s="2"/>
@@ -4621,11 +4446,11 @@
       <c r="Z88" s="2"/>
     </row>
     <row r="89" ht="14.25" customHeight="1">
-      <c r="A89" s="24"/>
-      <c r="B89" s="24"/>
-      <c r="C89" s="24"/>
-      <c r="D89" s="24"/>
-      <c r="E89" s="24"/>
+      <c r="A89" s="29"/>
+      <c r="B89" s="29"/>
+      <c r="C89" s="29"/>
+      <c r="D89" s="29"/>
+      <c r="E89" s="29"/>
       <c r="F89" s="2"/>
       <c r="G89" s="2"/>
       <c r="H89" s="2"/>
@@ -4649,11 +4474,11 @@
       <c r="Z89" s="2"/>
     </row>
     <row r="90" ht="14.25" customHeight="1">
-      <c r="A90" s="24"/>
-      <c r="B90" s="24"/>
-      <c r="C90" s="24"/>
-      <c r="D90" s="24"/>
-      <c r="E90" s="24"/>
+      <c r="A90" s="29"/>
+      <c r="B90" s="29"/>
+      <c r="C90" s="29"/>
+      <c r="D90" s="29"/>
+      <c r="E90" s="29"/>
       <c r="F90" s="2"/>
       <c r="G90" s="2"/>
       <c r="H90" s="2"/>
@@ -4677,11 +4502,11 @@
       <c r="Z90" s="2"/>
     </row>
     <row r="91" ht="14.25" customHeight="1">
-      <c r="A91" s="24"/>
-      <c r="B91" s="24"/>
-      <c r="C91" s="24"/>
-      <c r="D91" s="24"/>
-      <c r="E91" s="24"/>
+      <c r="A91" s="29"/>
+      <c r="B91" s="29"/>
+      <c r="C91" s="29"/>
+      <c r="D91" s="29"/>
+      <c r="E91" s="29"/>
       <c r="F91" s="2"/>
       <c r="G91" s="2"/>
       <c r="H91" s="2"/>
@@ -4705,11 +4530,11 @@
       <c r="Z91" s="2"/>
     </row>
     <row r="92" ht="14.25" customHeight="1">
-      <c r="A92" s="24"/>
-      <c r="B92" s="24"/>
-      <c r="C92" s="24"/>
-      <c r="D92" s="24"/>
-      <c r="E92" s="24"/>
+      <c r="A92" s="29"/>
+      <c r="B92" s="29"/>
+      <c r="C92" s="29"/>
+      <c r="D92" s="29"/>
+      <c r="E92" s="29"/>
       <c r="F92" s="2"/>
       <c r="G92" s="2"/>
       <c r="H92" s="2"/>
@@ -4733,11 +4558,11 @@
       <c r="Z92" s="2"/>
     </row>
     <row r="93" ht="14.25" customHeight="1">
-      <c r="A93" s="24"/>
-      <c r="B93" s="24"/>
-      <c r="C93" s="24"/>
-      <c r="D93" s="24"/>
-      <c r="E93" s="24"/>
+      <c r="A93" s="29"/>
+      <c r="B93" s="29"/>
+      <c r="C93" s="29"/>
+      <c r="D93" s="29"/>
+      <c r="E93" s="29"/>
       <c r="F93" s="2"/>
       <c r="G93" s="2"/>
       <c r="H93" s="2"/>
@@ -4761,11 +4586,11 @@
       <c r="Z93" s="2"/>
     </row>
     <row r="94" ht="14.25" customHeight="1">
-      <c r="A94" s="24"/>
-      <c r="B94" s="24"/>
-      <c r="C94" s="24"/>
-      <c r="D94" s="24"/>
-      <c r="E94" s="24"/>
+      <c r="A94" s="29"/>
+      <c r="B94" s="29"/>
+      <c r="C94" s="29"/>
+      <c r="D94" s="29"/>
+      <c r="E94" s="29"/>
       <c r="F94" s="2"/>
       <c r="G94" s="2"/>
       <c r="H94" s="2"/>
@@ -4789,11 +4614,11 @@
       <c r="Z94" s="2"/>
     </row>
     <row r="95" ht="14.25" customHeight="1">
-      <c r="A95" s="24"/>
-      <c r="B95" s="24"/>
-      <c r="C95" s="24"/>
-      <c r="D95" s="24"/>
-      <c r="E95" s="24"/>
+      <c r="A95" s="29"/>
+      <c r="B95" s="29"/>
+      <c r="C95" s="29"/>
+      <c r="D95" s="29"/>
+      <c r="E95" s="29"/>
       <c r="F95" s="2"/>
       <c r="G95" s="2"/>
       <c r="H95" s="2"/>
@@ -4817,11 +4642,11 @@
       <c r="Z95" s="2"/>
     </row>
     <row r="96" ht="14.25" customHeight="1">
-      <c r="A96" s="24"/>
-      <c r="B96" s="24"/>
-      <c r="C96" s="24"/>
-      <c r="D96" s="24"/>
-      <c r="E96" s="24"/>
+      <c r="A96" s="29"/>
+      <c r="B96" s="29"/>
+      <c r="C96" s="29"/>
+      <c r="D96" s="29"/>
+      <c r="E96" s="29"/>
       <c r="F96" s="2"/>
       <c r="G96" s="2"/>
       <c r="H96" s="2"/>
@@ -4845,11 +4670,11 @@
       <c r="Z96" s="2"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
-      <c r="A97" s="24"/>
-      <c r="B97" s="24"/>
-      <c r="C97" s="24"/>
-      <c r="D97" s="24"/>
-      <c r="E97" s="24"/>
+      <c r="A97" s="29"/>
+      <c r="B97" s="29"/>
+      <c r="C97" s="29"/>
+      <c r="D97" s="29"/>
+      <c r="E97" s="29"/>
       <c r="F97" s="2"/>
       <c r="G97" s="2"/>
       <c r="H97" s="2"/>
@@ -4873,11 +4698,11 @@
       <c r="Z97" s="2"/>
     </row>
     <row r="98" ht="14.25" customHeight="1">
-      <c r="A98" s="24"/>
-      <c r="B98" s="24"/>
-      <c r="C98" s="24"/>
-      <c r="D98" s="24"/>
-      <c r="E98" s="24"/>
+      <c r="A98" s="29"/>
+      <c r="B98" s="29"/>
+      <c r="C98" s="29"/>
+      <c r="D98" s="29"/>
+      <c r="E98" s="29"/>
       <c r="F98" s="2"/>
       <c r="G98" s="2"/>
       <c r="H98" s="2"/>
@@ -4901,11 +4726,11 @@
       <c r="Z98" s="2"/>
     </row>
     <row r="99" ht="14.25" customHeight="1">
-      <c r="A99" s="24"/>
-      <c r="B99" s="24"/>
-      <c r="C99" s="24"/>
-      <c r="D99" s="24"/>
-      <c r="E99" s="24"/>
+      <c r="A99" s="29"/>
+      <c r="B99" s="29"/>
+      <c r="C99" s="29"/>
+      <c r="D99" s="29"/>
+      <c r="E99" s="29"/>
       <c r="F99" s="2"/>
       <c r="G99" s="2"/>
       <c r="H99" s="2"/>
@@ -4929,11 +4754,11 @@
       <c r="Z99" s="2"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
-      <c r="A100" s="24"/>
-      <c r="B100" s="24"/>
-      <c r="C100" s="24"/>
-      <c r="D100" s="24"/>
-      <c r="E100" s="24"/>
+      <c r="A100" s="29"/>
+      <c r="B100" s="29"/>
+      <c r="C100" s="29"/>
+      <c r="D100" s="29"/>
+      <c r="E100" s="29"/>
       <c r="F100" s="2"/>
       <c r="G100" s="2"/>
       <c r="H100" s="2"/>
@@ -4957,11 +4782,11 @@
       <c r="Z100" s="2"/>
     </row>
     <row r="101" ht="14.25" customHeight="1">
-      <c r="A101" s="24"/>
-      <c r="B101" s="24"/>
-      <c r="C101" s="24"/>
-      <c r="D101" s="24"/>
-      <c r="E101" s="24"/>
+      <c r="A101" s="29"/>
+      <c r="B101" s="29"/>
+      <c r="C101" s="29"/>
+      <c r="D101" s="29"/>
+      <c r="E101" s="29"/>
       <c r="F101" s="2"/>
       <c r="G101" s="2"/>
       <c r="H101" s="2"/>
@@ -4985,11 +4810,11 @@
       <c r="Z101" s="2"/>
     </row>
     <row r="102" ht="14.25" customHeight="1">
-      <c r="A102" s="24"/>
-      <c r="B102" s="24"/>
-      <c r="C102" s="24"/>
-      <c r="D102" s="24"/>
-      <c r="E102" s="24"/>
+      <c r="A102" s="29"/>
+      <c r="B102" s="29"/>
+      <c r="C102" s="29"/>
+      <c r="D102" s="29"/>
+      <c r="E102" s="29"/>
       <c r="F102" s="2"/>
       <c r="G102" s="2"/>
       <c r="H102" s="2"/>
@@ -5013,11 +4838,11 @@
       <c r="Z102" s="2"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
-      <c r="A103" s="24"/>
-      <c r="B103" s="24"/>
-      <c r="C103" s="24"/>
-      <c r="D103" s="24"/>
-      <c r="E103" s="24"/>
+      <c r="A103" s="29"/>
+      <c r="B103" s="29"/>
+      <c r="C103" s="29"/>
+      <c r="D103" s="29"/>
+      <c r="E103" s="29"/>
       <c r="F103" s="2"/>
       <c r="G103" s="2"/>
       <c r="H103" s="2"/>
@@ -5041,11 +4866,11 @@
       <c r="Z103" s="2"/>
     </row>
     <row r="104" ht="14.25" customHeight="1">
-      <c r="A104" s="24"/>
-      <c r="B104" s="24"/>
-      <c r="C104" s="24"/>
-      <c r="D104" s="24"/>
-      <c r="E104" s="24"/>
+      <c r="A104" s="29"/>
+      <c r="B104" s="29"/>
+      <c r="C104" s="29"/>
+      <c r="D104" s="29"/>
+      <c r="E104" s="29"/>
       <c r="F104" s="2"/>
       <c r="G104" s="2"/>
       <c r="H104" s="2"/>
@@ -5069,11 +4894,11 @@
       <c r="Z104" s="2"/>
     </row>
     <row r="105" ht="14.25" customHeight="1">
-      <c r="A105" s="24"/>
-      <c r="B105" s="24"/>
-      <c r="C105" s="24"/>
-      <c r="D105" s="24"/>
-      <c r="E105" s="24"/>
+      <c r="A105" s="29"/>
+      <c r="B105" s="29"/>
+      <c r="C105" s="29"/>
+      <c r="D105" s="29"/>
+      <c r="E105" s="29"/>
       <c r="F105" s="2"/>
       <c r="G105" s="2"/>
       <c r="H105" s="2"/>
@@ -5097,11 +4922,11 @@
       <c r="Z105" s="2"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
-      <c r="A106" s="24"/>
-      <c r="B106" s="24"/>
-      <c r="C106" s="24"/>
-      <c r="D106" s="24"/>
-      <c r="E106" s="24"/>
+      <c r="A106" s="29"/>
+      <c r="B106" s="29"/>
+      <c r="C106" s="29"/>
+      <c r="D106" s="29"/>
+      <c r="E106" s="29"/>
       <c r="F106" s="2"/>
       <c r="G106" s="2"/>
       <c r="H106" s="2"/>
@@ -5125,11 +4950,11 @@
       <c r="Z106" s="2"/>
     </row>
     <row r="107" ht="14.25" customHeight="1">
-      <c r="A107" s="24"/>
-      <c r="B107" s="24"/>
-      <c r="C107" s="24"/>
-      <c r="D107" s="24"/>
-      <c r="E107" s="24"/>
+      <c r="A107" s="29"/>
+      <c r="B107" s="29"/>
+      <c r="C107" s="29"/>
+      <c r="D107" s="29"/>
+      <c r="E107" s="29"/>
       <c r="F107" s="2"/>
       <c r="G107" s="2"/>
       <c r="H107" s="2"/>
@@ -5153,11 +4978,11 @@
       <c r="Z107" s="2"/>
     </row>
     <row r="108" ht="14.25" customHeight="1">
-      <c r="A108" s="24"/>
-      <c r="B108" s="24"/>
-      <c r="C108" s="24"/>
-      <c r="D108" s="24"/>
-      <c r="E108" s="24"/>
+      <c r="A108" s="29"/>
+      <c r="B108" s="29"/>
+      <c r="C108" s="29"/>
+      <c r="D108" s="29"/>
+      <c r="E108" s="29"/>
       <c r="F108" s="2"/>
       <c r="G108" s="2"/>
       <c r="H108" s="2"/>
@@ -5181,11 +5006,11 @@
       <c r="Z108" s="2"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
-      <c r="A109" s="24"/>
-      <c r="B109" s="24"/>
-      <c r="C109" s="24"/>
-      <c r="D109" s="24"/>
-      <c r="E109" s="24"/>
+      <c r="A109" s="29"/>
+      <c r="B109" s="29"/>
+      <c r="C109" s="29"/>
+      <c r="D109" s="29"/>
+      <c r="E109" s="29"/>
       <c r="F109" s="2"/>
       <c r="G109" s="2"/>
       <c r="H109" s="2"/>
@@ -5209,11 +5034,11 @@
       <c r="Z109" s="2"/>
     </row>
     <row r="110" ht="14.25" customHeight="1">
-      <c r="A110" s="24"/>
-      <c r="B110" s="24"/>
-      <c r="C110" s="24"/>
-      <c r="D110" s="24"/>
-      <c r="E110" s="24"/>
+      <c r="A110" s="29"/>
+      <c r="B110" s="29"/>
+      <c r="C110" s="29"/>
+      <c r="D110" s="29"/>
+      <c r="E110" s="29"/>
       <c r="F110" s="2"/>
       <c r="G110" s="2"/>
       <c r="H110" s="2"/>
@@ -5237,11 +5062,11 @@
       <c r="Z110" s="2"/>
     </row>
     <row r="111" ht="14.25" customHeight="1">
-      <c r="A111" s="24"/>
-      <c r="B111" s="24"/>
-      <c r="C111" s="24"/>
-      <c r="D111" s="24"/>
-      <c r="E111" s="24"/>
+      <c r="A111" s="29"/>
+      <c r="B111" s="29"/>
+      <c r="C111" s="29"/>
+      <c r="D111" s="29"/>
+      <c r="E111" s="29"/>
       <c r="F111" s="2"/>
       <c r="G111" s="2"/>
       <c r="H111" s="2"/>
@@ -5265,11 +5090,11 @@
       <c r="Z111" s="2"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
-      <c r="A112" s="24"/>
-      <c r="B112" s="24"/>
-      <c r="C112" s="24"/>
-      <c r="D112" s="24"/>
-      <c r="E112" s="24"/>
+      <c r="A112" s="29"/>
+      <c r="B112" s="29"/>
+      <c r="C112" s="29"/>
+      <c r="D112" s="29"/>
+      <c r="E112" s="29"/>
       <c r="F112" s="2"/>
       <c r="G112" s="2"/>
       <c r="H112" s="2"/>
@@ -5293,11 +5118,11 @@
       <c r="Z112" s="2"/>
     </row>
     <row r="113" ht="14.25" customHeight="1">
-      <c r="A113" s="24"/>
-      <c r="B113" s="24"/>
-      <c r="C113" s="24"/>
-      <c r="D113" s="24"/>
-      <c r="E113" s="24"/>
+      <c r="A113" s="29"/>
+      <c r="B113" s="29"/>
+      <c r="C113" s="29"/>
+      <c r="D113" s="29"/>
+      <c r="E113" s="29"/>
       <c r="F113" s="2"/>
       <c r="G113" s="2"/>
       <c r="H113" s="2"/>
@@ -5321,11 +5146,11 @@
       <c r="Z113" s="2"/>
     </row>
     <row r="114" ht="14.25" customHeight="1">
-      <c r="A114" s="24"/>
-      <c r="B114" s="24"/>
-      <c r="C114" s="24"/>
-      <c r="D114" s="24"/>
-      <c r="E114" s="24"/>
+      <c r="A114" s="29"/>
+      <c r="B114" s="29"/>
+      <c r="C114" s="29"/>
+      <c r="D114" s="29"/>
+      <c r="E114" s="29"/>
       <c r="F114" s="2"/>
       <c r="G114" s="2"/>
       <c r="H114" s="2"/>
@@ -5349,11 +5174,11 @@
       <c r="Z114" s="2"/>
     </row>
     <row r="115" ht="14.25" customHeight="1">
-      <c r="A115" s="24"/>
-      <c r="B115" s="24"/>
-      <c r="C115" s="24"/>
-      <c r="D115" s="24"/>
-      <c r="E115" s="24"/>
+      <c r="A115" s="29"/>
+      <c r="B115" s="29"/>
+      <c r="C115" s="29"/>
+      <c r="D115" s="29"/>
+      <c r="E115" s="29"/>
       <c r="F115" s="2"/>
       <c r="G115" s="2"/>
       <c r="H115" s="2"/>
@@ -5377,11 +5202,11 @@
       <c r="Z115" s="2"/>
     </row>
     <row r="116" ht="14.25" customHeight="1">
-      <c r="A116" s="24"/>
-      <c r="B116" s="24"/>
-      <c r="C116" s="24"/>
-      <c r="D116" s="24"/>
-      <c r="E116" s="24"/>
+      <c r="A116" s="2"/>
+      <c r="B116" s="2"/>
+      <c r="C116" s="2"/>
+      <c r="D116" s="2"/>
+      <c r="E116" s="2"/>
       <c r="F116" s="2"/>
       <c r="G116" s="2"/>
       <c r="H116" s="2"/>
@@ -5405,11 +5230,11 @@
       <c r="Z116" s="2"/>
     </row>
     <row r="117" ht="14.25" customHeight="1">
-      <c r="A117" s="24"/>
-      <c r="B117" s="24"/>
-      <c r="C117" s="24"/>
-      <c r="D117" s="24"/>
-      <c r="E117" s="24"/>
+      <c r="A117" s="2"/>
+      <c r="B117" s="2"/>
+      <c r="C117" s="2"/>
+      <c r="D117" s="2"/>
+      <c r="E117" s="2"/>
       <c r="F117" s="2"/>
       <c r="G117" s="2"/>
       <c r="H117" s="2"/>
@@ -5433,11 +5258,11 @@
       <c r="Z117" s="2"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
-      <c r="A118" s="24"/>
-      <c r="B118" s="24"/>
-      <c r="C118" s="24"/>
-      <c r="D118" s="24"/>
-      <c r="E118" s="24"/>
+      <c r="A118" s="2"/>
+      <c r="B118" s="2"/>
+      <c r="C118" s="2"/>
+      <c r="D118" s="2"/>
+      <c r="E118" s="2"/>
       <c r="F118" s="2"/>
       <c r="G118" s="2"/>
       <c r="H118" s="2"/>
@@ -5461,11 +5286,11 @@
       <c r="Z118" s="2"/>
     </row>
     <row r="119" ht="14.25" customHeight="1">
-      <c r="A119" s="24"/>
-      <c r="B119" s="24"/>
-      <c r="C119" s="24"/>
-      <c r="D119" s="24"/>
-      <c r="E119" s="24"/>
+      <c r="A119" s="2"/>
+      <c r="B119" s="2"/>
+      <c r="C119" s="2"/>
+      <c r="D119" s="2"/>
+      <c r="E119" s="2"/>
       <c r="F119" s="2"/>
       <c r="G119" s="2"/>
       <c r="H119" s="2"/>
@@ -5489,11 +5314,11 @@
       <c r="Z119" s="2"/>
     </row>
     <row r="120" ht="14.25" customHeight="1">
-      <c r="A120" s="24"/>
-      <c r="B120" s="24"/>
-      <c r="C120" s="24"/>
-      <c r="D120" s="24"/>
-      <c r="E120" s="24"/>
+      <c r="A120" s="2"/>
+      <c r="B120" s="2"/>
+      <c r="C120" s="2"/>
+      <c r="D120" s="2"/>
+      <c r="E120" s="2"/>
       <c r="F120" s="2"/>
       <c r="G120" s="2"/>
       <c r="H120" s="2"/>
@@ -5517,11 +5342,11 @@
       <c r="Z120" s="2"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
-      <c r="A121" s="24"/>
-      <c r="B121" s="24"/>
-      <c r="C121" s="24"/>
-      <c r="D121" s="24"/>
-      <c r="E121" s="24"/>
+      <c r="A121" s="2"/>
+      <c r="B121" s="2"/>
+      <c r="C121" s="2"/>
+      <c r="D121" s="2"/>
+      <c r="E121" s="2"/>
       <c r="F121" s="2"/>
       <c r="G121" s="2"/>
       <c r="H121" s="2"/>
@@ -5545,11 +5370,11 @@
       <c r="Z121" s="2"/>
     </row>
     <row r="122" ht="14.25" customHeight="1">
-      <c r="A122" s="24"/>
-      <c r="B122" s="24"/>
-      <c r="C122" s="24"/>
-      <c r="D122" s="24"/>
-      <c r="E122" s="24"/>
+      <c r="A122" s="2"/>
+      <c r="B122" s="2"/>
+      <c r="C122" s="2"/>
+      <c r="D122" s="2"/>
+      <c r="E122" s="2"/>
       <c r="F122" s="2"/>
       <c r="G122" s="2"/>
       <c r="H122" s="2"/>
@@ -29764,206 +29589,11 @@
       <c r="Y986" s="2"/>
       <c r="Z986" s="2"/>
     </row>
-    <row r="987" ht="14.25" customHeight="1">
-      <c r="A987" s="2"/>
-      <c r="B987" s="2"/>
-      <c r="C987" s="2"/>
-      <c r="D987" s="2"/>
-      <c r="E987" s="2"/>
-      <c r="F987" s="2"/>
-      <c r="G987" s="2"/>
-      <c r="H987" s="2"/>
-      <c r="I987" s="2"/>
-      <c r="J987" s="2"/>
-      <c r="K987" s="2"/>
-      <c r="L987" s="2"/>
-      <c r="M987" s="2"/>
-      <c r="N987" s="2"/>
-      <c r="O987" s="2"/>
-      <c r="P987" s="2"/>
-      <c r="Q987" s="2"/>
-      <c r="R987" s="2"/>
-      <c r="S987" s="2"/>
-      <c r="T987" s="2"/>
-      <c r="U987" s="2"/>
-      <c r="V987" s="2"/>
-      <c r="W987" s="2"/>
-      <c r="X987" s="2"/>
-      <c r="Y987" s="2"/>
-      <c r="Z987" s="2"/>
-    </row>
-    <row r="988" ht="14.25" customHeight="1">
-      <c r="A988" s="2"/>
-      <c r="B988" s="2"/>
-      <c r="C988" s="2"/>
-      <c r="D988" s="2"/>
-      <c r="E988" s="2"/>
-      <c r="F988" s="2"/>
-      <c r="G988" s="2"/>
-      <c r="H988" s="2"/>
-      <c r="I988" s="2"/>
-      <c r="J988" s="2"/>
-      <c r="K988" s="2"/>
-      <c r="L988" s="2"/>
-      <c r="M988" s="2"/>
-      <c r="N988" s="2"/>
-      <c r="O988" s="2"/>
-      <c r="P988" s="2"/>
-      <c r="Q988" s="2"/>
-      <c r="R988" s="2"/>
-      <c r="S988" s="2"/>
-      <c r="T988" s="2"/>
-      <c r="U988" s="2"/>
-      <c r="V988" s="2"/>
-      <c r="W988" s="2"/>
-      <c r="X988" s="2"/>
-      <c r="Y988" s="2"/>
-      <c r="Z988" s="2"/>
-    </row>
-    <row r="989" ht="14.25" customHeight="1">
-      <c r="A989" s="2"/>
-      <c r="B989" s="2"/>
-      <c r="C989" s="2"/>
-      <c r="D989" s="2"/>
-      <c r="E989" s="2"/>
-      <c r="F989" s="2"/>
-      <c r="G989" s="2"/>
-      <c r="H989" s="2"/>
-      <c r="I989" s="2"/>
-      <c r="J989" s="2"/>
-      <c r="K989" s="2"/>
-      <c r="L989" s="2"/>
-      <c r="M989" s="2"/>
-      <c r="N989" s="2"/>
-      <c r="O989" s="2"/>
-      <c r="P989" s="2"/>
-      <c r="Q989" s="2"/>
-      <c r="R989" s="2"/>
-      <c r="S989" s="2"/>
-      <c r="T989" s="2"/>
-      <c r="U989" s="2"/>
-      <c r="V989" s="2"/>
-      <c r="W989" s="2"/>
-      <c r="X989" s="2"/>
-      <c r="Y989" s="2"/>
-      <c r="Z989" s="2"/>
-    </row>
-    <row r="990" ht="14.25" customHeight="1">
-      <c r="A990" s="2"/>
-      <c r="B990" s="2"/>
-      <c r="C990" s="2"/>
-      <c r="D990" s="2"/>
-      <c r="E990" s="2"/>
-      <c r="F990" s="2"/>
-      <c r="G990" s="2"/>
-      <c r="H990" s="2"/>
-      <c r="I990" s="2"/>
-      <c r="J990" s="2"/>
-      <c r="K990" s="2"/>
-      <c r="L990" s="2"/>
-      <c r="M990" s="2"/>
-      <c r="N990" s="2"/>
-      <c r="O990" s="2"/>
-      <c r="P990" s="2"/>
-      <c r="Q990" s="2"/>
-      <c r="R990" s="2"/>
-      <c r="S990" s="2"/>
-      <c r="T990" s="2"/>
-      <c r="U990" s="2"/>
-      <c r="V990" s="2"/>
-      <c r="W990" s="2"/>
-      <c r="X990" s="2"/>
-      <c r="Y990" s="2"/>
-      <c r="Z990" s="2"/>
-    </row>
-    <row r="991" ht="14.25" customHeight="1">
-      <c r="A991" s="2"/>
-      <c r="B991" s="2"/>
-      <c r="C991" s="2"/>
-      <c r="D991" s="2"/>
-      <c r="E991" s="2"/>
-      <c r="F991" s="2"/>
-      <c r="G991" s="2"/>
-      <c r="H991" s="2"/>
-      <c r="I991" s="2"/>
-      <c r="J991" s="2"/>
-      <c r="K991" s="2"/>
-      <c r="L991" s="2"/>
-      <c r="M991" s="2"/>
-      <c r="N991" s="2"/>
-      <c r="O991" s="2"/>
-      <c r="P991" s="2"/>
-      <c r="Q991" s="2"/>
-      <c r="R991" s="2"/>
-      <c r="S991" s="2"/>
-      <c r="T991" s="2"/>
-      <c r="U991" s="2"/>
-      <c r="V991" s="2"/>
-      <c r="W991" s="2"/>
-      <c r="X991" s="2"/>
-      <c r="Y991" s="2"/>
-      <c r="Z991" s="2"/>
-    </row>
-    <row r="992" ht="14.25" customHeight="1">
-      <c r="A992" s="2"/>
-      <c r="B992" s="2"/>
-      <c r="C992" s="2"/>
-      <c r="D992" s="2"/>
-      <c r="E992" s="2"/>
-      <c r="F992" s="2"/>
-      <c r="G992" s="2"/>
-      <c r="H992" s="2"/>
-      <c r="I992" s="2"/>
-      <c r="J992" s="2"/>
-      <c r="K992" s="2"/>
-      <c r="L992" s="2"/>
-      <c r="M992" s="2"/>
-      <c r="N992" s="2"/>
-      <c r="O992" s="2"/>
-      <c r="P992" s="2"/>
-      <c r="Q992" s="2"/>
-      <c r="R992" s="2"/>
-      <c r="S992" s="2"/>
-      <c r="T992" s="2"/>
-      <c r="U992" s="2"/>
-      <c r="V992" s="2"/>
-      <c r="W992" s="2"/>
-      <c r="X992" s="2"/>
-      <c r="Y992" s="2"/>
-      <c r="Z992" s="2"/>
-    </row>
-    <row r="993" ht="14.25" customHeight="1">
-      <c r="A993" s="2"/>
-      <c r="B993" s="2"/>
-      <c r="C993" s="2"/>
-      <c r="D993" s="2"/>
-      <c r="E993" s="2"/>
-      <c r="F993" s="2"/>
-      <c r="G993" s="2"/>
-      <c r="H993" s="2"/>
-      <c r="I993" s="2"/>
-      <c r="J993" s="2"/>
-      <c r="K993" s="2"/>
-      <c r="L993" s="2"/>
-      <c r="M993" s="2"/>
-      <c r="N993" s="2"/>
-      <c r="O993" s="2"/>
-      <c r="P993" s="2"/>
-      <c r="Q993" s="2"/>
-      <c r="R993" s="2"/>
-      <c r="S993" s="2"/>
-      <c r="T993" s="2"/>
-      <c r="U993" s="2"/>
-      <c r="V993" s="2"/>
-      <c r="W993" s="2"/>
-      <c r="X993" s="2"/>
-      <c r="Y993" s="2"/>
-      <c r="Z993" s="2"/>
-    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="D1:F3"/>
-    <mergeCell ref="I55:J55"/>
+    <mergeCell ref="I48:J48"/>
+    <mergeCell ref="I49:J49"/>
   </mergeCells>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.699305555555556" right="0.699305555555556" top="0.75"/>

</xml_diff>